<commit_message>
feat: sinkronkan kelas pengguna & anggota, input buku tamu manual, fitur naik kelas, wajib keterangan penolakan & pinjam ulang, pencarian nama/NISN sirkulasi, bulk approve/reject/terima, dan filter limit data
</commit_message>
<xml_diff>
--- a/public/template_pengguna.xlsx
+++ b/public/template_pengguna.xlsx
@@ -1,70 +1,101 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79CBD53B-9459-4238-BC49-B39F1FD94036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Template Pengguna" sheetId="1" r:id="rId1"/>
+    <sheet name="Template Pengguna" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="7">
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>username</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>Jane Smith</t>
-  </si>
-  <si>
-    <t>Agus Rudi</t>
-  </si>
-  <si>
-    <t>NISN</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
+  <si>
+    <t>Nama</t>
+  </si>
+  <si>
+    <t>Username/NISN</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Kelas</t>
+  </si>
+  <si>
+    <t>Ahmad Fauzi</t>
+  </si>
+  <si>
+    <t>0012345678</t>
+  </si>
+  <si>
+    <t>X IPA 1</t>
+  </si>
+  <si>
+    <t>Siti Nurhaliza</t>
+  </si>
+  <si>
+    <t>0012345679</t>
+  </si>
+  <si>
+    <t>X IPS 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="1"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF808080"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -72,26 +103,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -170,6 +212,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -204,6 +247,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -379,58 +423,64 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="2" width="14.6328125" customWidth="1"/>
+    <col min="1" max="1" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="9.283" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
+    <row r="3" spans="1:4">
+      <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>